<commit_message>
csvtoexcel also seems to work
</commit_message>
<xml_diff>
--- a/results_clean.xlsx
+++ b/results_clean.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Results" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results'!$A$1:$K$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results'!$A$1:$K$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -24,16 +24,13 @@
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="yyyy-mm-dd hh:mm:ss"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -44,7 +41,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -52,21 +49,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -435,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -452,91 +440,91 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>x1</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>y1</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>x2</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>y2</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>x3</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>y3</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>angle</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>energy_objective</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>stress_constraint</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>best_in_file</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="1" t="n">
         <v>16.66845732846889</v>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B2" s="1" t="n">
         <v>14.90057320001673</v>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C2" s="1" t="n">
         <v>38.86381047832207</v>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" s="1" t="n">
         <v>10.03832842036743</v>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" s="1" t="n">
         <v>28.36416089100964</v>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="F2" s="1" t="n">
         <v>48.73969842501265</v>
       </c>
-      <c r="G2" s="2" t="n">
+      <c r="G2" s="1" t="n">
         <v>3.060667775754733</v>
       </c>
-      <c r="H2" s="3" t="n">
+      <c r="H2" s="2" t="n">
         <v>13183.1783488889</v>
       </c>
-      <c r="I2" s="3" t="n">
+      <c r="I2" s="2" t="n">
         <v>229.039</v>
       </c>
-      <c r="J2" s="4" t="n">
+      <c r="J2" s="3" t="n">
         <v>46182.78790509259</v>
       </c>
       <c r="K2" t="b">
@@ -544,34 +532,34 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="1" t="n">
         <v>13.78471682985224</v>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B3" s="1" t="n">
         <v>16.21393024762252</v>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="C3" s="1" t="n">
         <v>10.59325996569644</v>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D3" s="1" t="n">
         <v>36.06356980491166</v>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" s="1" t="n">
         <v>36.07082245901849</v>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="F3" s="1" t="n">
         <v>28.55955393861952</v>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="G3" s="1" t="n">
         <v>76.96268176577249</v>
       </c>
-      <c r="H3" s="3" t="n">
+      <c r="H3" s="2" t="n">
         <v>13091.41425410255</v>
       </c>
-      <c r="I3" s="3" t="n">
+      <c r="I3" s="2" t="n">
         <v>234.9595</v>
       </c>
-      <c r="J3" s="4" t="n">
+      <c r="J3" s="3" t="n">
         <v>46181.58004629629</v>
       </c>
       <c r="K3" t="b">
@@ -579,34 +567,34 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="1" t="n">
         <v>17.79972151146293</v>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B4" s="1" t="n">
         <v>17.69341384342146</v>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" s="1" t="n">
         <v>46.48075530504345</v>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D4" s="1" t="n">
         <v>9.328346721716176</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="1" t="n">
         <v>32.18668778246325</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="1" t="n">
         <v>45.74821535730867</v>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="G4" s="1" t="n">
         <v>6.445466519477314</v>
       </c>
-      <c r="H4" s="3" t="n">
+      <c r="H4" s="2" t="n">
         <v>13084.58563732278</v>
       </c>
-      <c r="I4" s="3" t="n">
+      <c r="I4" s="2" t="n">
         <v>234.54925</v>
       </c>
-      <c r="J4" s="4" t="n">
+      <c r="J4" s="3" t="n">
         <v>46182.76752314815</v>
       </c>
       <c r="K4" t="b">
@@ -614,34 +602,34 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="1" t="n">
         <v>17.58736126294788</v>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B5" s="1" t="n">
         <v>16.45887634010303</v>
       </c>
-      <c r="C5" s="2" t="n">
+      <c r="C5" s="1" t="n">
         <v>47.45352527302221</v>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="D5" s="1" t="n">
         <v>8.576653324750513</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="1" t="n">
         <v>32.82334208094247</v>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="F5" s="1" t="n">
         <v>46.745392166702</v>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="G5" s="1" t="n">
         <v>7.732490961886047</v>
       </c>
-      <c r="H5" s="3" t="n">
+      <c r="H5" s="2" t="n">
         <v>13073.63342736011</v>
       </c>
-      <c r="I5" s="3" t="n">
+      <c r="I5" s="2" t="n">
         <v>230.39875</v>
       </c>
-      <c r="J5" s="4" t="n">
+      <c r="J5" s="3" t="n">
         <v>46182.15122685185</v>
       </c>
       <c r="K5" t="b">
@@ -649,34 +637,34 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="1" t="n">
         <v>13.71791013779612</v>
       </c>
-      <c r="B6" s="2" t="n">
+      <c r="B6" s="1" t="n">
         <v>18.10904520314511</v>
       </c>
-      <c r="C6" s="2" t="n">
+      <c r="C6" s="1" t="n">
         <v>10.92071189213304</v>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D6" s="1" t="n">
         <v>36.6622583775164</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" s="1" t="n">
         <v>36.41744258847353</v>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="F6" s="1" t="n">
         <v>27.51048220857797</v>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="G6" s="1" t="n">
         <v>75.74096458387024</v>
       </c>
-      <c r="H6" s="3" t="n">
+      <c r="H6" s="2" t="n">
         <v>13071.57609008536</v>
       </c>
-      <c r="I6" s="3" t="n">
+      <c r="I6" s="2" t="n">
         <v>232.0765</v>
       </c>
-      <c r="J6" s="4" t="n">
+      <c r="J6" s="3" t="n">
         <v>46182.68601851852</v>
       </c>
       <c r="K6" t="b">
@@ -684,34 +672,34 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="1" t="n">
         <v>41.8658806151136</v>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B7" s="1" t="n">
         <v>15.37870830271605</v>
       </c>
-      <c r="C7" s="2" t="n">
+      <c r="C7" s="1" t="n">
         <v>23.27808313388434</v>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="D7" s="1" t="n">
         <v>17.76876422795642</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="1" t="n">
         <v>32.80848986515946</v>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="F7" s="1" t="n">
         <v>49.56039126315637</v>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="G7" s="1" t="n">
         <v>4.004847201307703</v>
       </c>
-      <c r="H7" s="3" t="n">
+      <c r="H7" s="2" t="n">
         <v>13041.49585837179</v>
       </c>
-      <c r="I7" s="3" t="n">
+      <c r="I7" s="2" t="n">
         <v>235.48675</v>
       </c>
-      <c r="J7" s="4" t="n">
+      <c r="J7" s="3" t="n">
         <v>46181.61930555556</v>
       </c>
       <c r="K7" t="b">
@@ -719,34 +707,34 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="1" t="n">
         <v>15.76699354991495</v>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B8" s="1" t="n">
         <v>17.34416185704958</v>
       </c>
-      <c r="C8" s="2" t="n">
+      <c r="C8" s="1" t="n">
         <v>36.82264430163571</v>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="D8" s="1" t="n">
         <v>20.82884517757701</v>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="1" t="n">
         <v>27.54321199229494</v>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="F8" s="1" t="n">
         <v>43.12916308199385</v>
       </c>
-      <c r="G8" s="2" t="n">
+      <c r="G8" s="1" t="n">
         <v>4.382860985545683</v>
       </c>
-      <c r="H8" s="3" t="n">
+      <c r="H8" s="2" t="n">
         <v>13039.54099967359</v>
       </c>
-      <c r="I8" s="3" t="n">
+      <c r="I8" s="2" t="n">
         <v>232.88425</v>
       </c>
-      <c r="J8" s="4" t="n">
+      <c r="J8" s="3" t="n">
         <v>46182.61533564814</v>
       </c>
       <c r="K8" t="b">
@@ -754,34 +742,34 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="1" t="n">
         <v>12.63807670451446</v>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B9" s="1" t="n">
         <v>15.95744954515774</v>
       </c>
-      <c r="C9" s="2" t="n">
+      <c r="C9" s="1" t="n">
         <v>35.69464860799762</v>
       </c>
-      <c r="D9" s="2" t="n">
+      <c r="D9" s="1" t="n">
         <v>12.31185540225469</v>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" s="1" t="n">
         <v>27.67290769582389</v>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="F9" s="1" t="n">
         <v>39.58733460632672</v>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="G9" s="1" t="n">
         <v>15.28166470319942</v>
       </c>
-      <c r="H9" s="3" t="n">
+      <c r="H9" s="2" t="n">
         <v>13030.88753714936</v>
       </c>
-      <c r="I9" s="3" t="n">
+      <c r="I9" s="2" t="n">
         <v>233.16625</v>
       </c>
-      <c r="J9" s="4" t="n">
+      <c r="J9" s="3" t="n">
         <v>46182.59353009259</v>
       </c>
       <c r="K9" t="b">
@@ -789,34 +777,34 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="1" t="n">
         <v>16.63370127960484</v>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="B10" s="1" t="n">
         <v>15.5698375808045</v>
       </c>
-      <c r="C10" s="2" t="n">
+      <c r="C10" s="1" t="n">
         <v>44.61368353212431</v>
       </c>
-      <c r="D10" s="2" t="n">
+      <c r="D10" s="1" t="n">
         <v>8.10871062925712</v>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E10" s="1" t="n">
         <v>33.48757536800954</v>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="F10" s="1" t="n">
         <v>47.40549517830886</v>
       </c>
-      <c r="G10" s="2" t="n">
+      <c r="G10" s="1" t="n">
         <v>6.080468056109986</v>
       </c>
-      <c r="H10" s="3" t="n">
+      <c r="H10" s="2" t="n">
         <v>13024.42830290779</v>
       </c>
-      <c r="I10" s="3" t="n">
+      <c r="I10" s="2" t="n">
         <v>243.60925</v>
       </c>
-      <c r="J10" s="4" t="n">
+      <c r="J10" s="3" t="n">
         <v>46182.57434027778</v>
       </c>
       <c r="K10" t="b">
@@ -824,34 +812,34 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="1" t="n">
         <v>17.25260165231997</v>
       </c>
-      <c r="B11" s="2" t="n">
+      <c r="B11" s="1" t="n">
         <v>18.21456551879732</v>
       </c>
-      <c r="C11" s="2" t="n">
+      <c r="C11" s="1" t="n">
         <v>11.29227638693606</v>
       </c>
-      <c r="D11" s="2" t="n">
+      <c r="D11" s="1" t="n">
         <v>37.72302288323579</v>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="E11" s="1" t="n">
         <v>40.53305602737925</v>
       </c>
-      <c r="F11" s="2" t="n">
+      <c r="F11" s="1" t="n">
         <v>30.1222227565979</v>
       </c>
-      <c r="G11" s="2" t="n">
+      <c r="G11" s="1" t="n">
         <v>73.05607094516266</v>
       </c>
-      <c r="H11" s="3" t="n">
+      <c r="H11" s="2" t="n">
         <v>12999.09867980331</v>
       </c>
-      <c r="I11" s="3" t="n">
+      <c r="I11" s="2" t="n">
         <v>239.53525</v>
       </c>
-      <c r="J11" s="4" t="n">
+      <c r="J11" s="3" t="n">
         <v>46182.60178240741</v>
       </c>
       <c r="K11" t="b">
@@ -859,34 +847,34 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="1" t="n">
         <v>43.56368398257163</v>
       </c>
-      <c r="B12" s="2" t="n">
+      <c r="B12" s="1" t="n">
         <v>15.15588461720007</v>
       </c>
-      <c r="C12" s="2" t="n">
+      <c r="C12" s="1" t="n">
         <v>22.29902711583871</v>
       </c>
-      <c r="D12" s="2" t="n">
+      <c r="D12" s="1" t="n">
         <v>20.43515019017654</v>
       </c>
-      <c r="E12" s="2" t="n">
+      <c r="E12" s="1" t="n">
         <v>33.88465155652464</v>
       </c>
-      <c r="F12" s="2" t="n">
+      <c r="F12" s="1" t="n">
         <v>48.75409190845778</v>
       </c>
-      <c r="G12" s="2" t="n">
+      <c r="G12" s="1" t="n">
         <v>3.423824078511241</v>
       </c>
-      <c r="H12" s="3" t="n">
+      <c r="H12" s="2" t="n">
         <v>12985.98554837028</v>
       </c>
-      <c r="I12" s="3" t="n">
+      <c r="I12" s="2" t="n">
         <v>233.1355</v>
       </c>
-      <c r="J12" s="4" t="n">
+      <c r="J12" s="3" t="n">
         <v>46182.52965277778</v>
       </c>
       <c r="K12" t="b">
@@ -894,34 +882,34 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="1" t="n">
         <v>17.94757986531874</v>
       </c>
-      <c r="B13" s="2" t="n">
+      <c r="B13" s="1" t="n">
         <v>16.84469598424037</v>
       </c>
-      <c r="C13" s="2" t="n">
+      <c r="C13" s="1" t="n">
         <v>51.00723850792093</v>
       </c>
-      <c r="D13" s="2" t="n">
+      <c r="D13" s="1" t="n">
         <v>44.32329678834844</v>
       </c>
-      <c r="E13" s="2" t="n">
+      <c r="E13" s="1" t="n">
         <v>39.51561233856795</v>
       </c>
-      <c r="F13" s="2" t="n">
+      <c r="F13" s="1" t="n">
         <v>34.18006619235404</v>
       </c>
-      <c r="G13" s="2" t="n">
+      <c r="G13" s="1" t="n">
         <v>49.58832168563249</v>
       </c>
-      <c r="H13" s="3" t="n">
+      <c r="H13" s="2" t="n">
         <v>12926.78503231161</v>
       </c>
-      <c r="I13" s="3" t="n">
+      <c r="I13" s="2" t="n">
         <v>261.9415</v>
       </c>
-      <c r="J13" s="4" t="n">
+      <c r="J13" s="3" t="n">
         <v>46182.52229166667</v>
       </c>
       <c r="K13" t="b">
@@ -929,34 +917,34 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="1" t="n">
         <v>11.26262399697765</v>
       </c>
-      <c r="B14" s="2" t="n">
+      <c r="B14" s="1" t="n">
         <v>14.7745708576305</v>
       </c>
-      <c r="C14" s="2" t="n">
+      <c r="C14" s="1" t="n">
         <v>44.19256877440593</v>
       </c>
-      <c r="D14" s="2" t="n">
+      <c r="D14" s="1" t="n">
         <v>14.75265751951711</v>
       </c>
-      <c r="E14" s="2" t="n">
+      <c r="E14" s="1" t="n">
         <v>31.50532968846312</v>
       </c>
-      <c r="F14" s="2" t="n">
+      <c r="F14" s="1" t="n">
         <v>46.90990440494782</v>
       </c>
-      <c r="G14" s="2" t="n">
+      <c r="G14" s="1" t="n">
         <v>3.800946599292743</v>
       </c>
-      <c r="H14" s="3" t="n">
+      <c r="H14" s="2" t="n">
         <v>12912.77360106467</v>
       </c>
-      <c r="I14" s="3" t="n">
+      <c r="I14" s="2" t="n">
         <v>234.91</v>
       </c>
-      <c r="J14" s="4" t="n">
+      <c r="J14" s="3" t="n">
         <v>46182.55270833334</v>
       </c>
       <c r="K14" t="b">
@@ -964,34 +952,34 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n">
+      <c r="A15" s="1" t="n">
         <v>13.33934470733688</v>
       </c>
-      <c r="B15" s="2" t="n">
+      <c r="B15" s="1" t="n">
         <v>16.92409346141374</v>
       </c>
-      <c r="C15" s="2" t="n">
+      <c r="C15" s="1" t="n">
         <v>36.19215939817842</v>
       </c>
-      <c r="D15" s="2" t="n">
+      <c r="D15" s="1" t="n">
         <v>14.53122691792867</v>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="E15" s="1" t="n">
         <v>28.83171218130013</v>
       </c>
-      <c r="F15" s="2" t="n">
+      <c r="F15" s="1" t="n">
         <v>38.49906907960096</v>
       </c>
-      <c r="G15" s="2" t="n">
+      <c r="G15" s="1" t="n">
         <v>11.29812525550822</v>
       </c>
-      <c r="H15" s="3" t="n">
+      <c r="H15" s="2" t="n">
         <v>12887.47232061737</v>
       </c>
-      <c r="I15" s="3" t="n">
+      <c r="I15" s="2" t="n">
         <v>249.622</v>
       </c>
-      <c r="J15" s="4" t="n">
+      <c r="J15" s="3" t="n">
         <v>46182.563125</v>
       </c>
       <c r="K15" t="b">
@@ -999,34 +987,34 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
+      <c r="A16" s="1" t="n">
         <v>15.626117785012</v>
       </c>
-      <c r="B16" s="2" t="n">
+      <c r="B16" s="1" t="n">
         <v>13.97537155172789</v>
       </c>
-      <c r="C16" s="2" t="n">
+      <c r="C16" s="1" t="n">
         <v>32.83268303598197</v>
       </c>
-      <c r="D16" s="2" t="n">
+      <c r="D16" s="1" t="n">
         <v>8.326124531530141</v>
       </c>
-      <c r="E16" s="2" t="n">
+      <c r="E16" s="1" t="n">
         <v>34.81057894851994</v>
       </c>
-      <c r="F16" s="2" t="n">
+      <c r="F16" s="1" t="n">
         <v>42.38662545986336</v>
       </c>
-      <c r="G16" s="2" t="n">
+      <c r="G16" s="1" t="n">
         <v>28.00450830446921</v>
       </c>
-      <c r="H16" s="3" t="n">
+      <c r="H16" s="2" t="n">
         <v>12634.1080121104</v>
       </c>
-      <c r="I16" s="3" t="n">
+      <c r="I16" s="2" t="n">
         <v>267.10675</v>
       </c>
-      <c r="J16" s="4" t="n">
+      <c r="J16" s="3" t="n">
         <v>46182.05643518519</v>
       </c>
       <c r="K16" t="b">
@@ -1034,42 +1022,77 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
+      <c r="A17" s="1" t="n">
+        <v>15.25529519300532</v>
+      </c>
+      <c r="B17" s="1" t="n">
+        <v>12.11419195930596</v>
+      </c>
+      <c r="C17" s="1" t="n">
+        <v>10.05183024601476</v>
+      </c>
+      <c r="D17" s="1" t="n">
+        <v>43.97564648706527</v>
+      </c>
+      <c r="E17" s="1" t="n">
+        <v>46.09898454414606</v>
+      </c>
+      <c r="F17" s="1" t="n">
+        <v>35.73229378624028</v>
+      </c>
+      <c r="G17" s="1" t="n">
+        <v>73.32411555469949</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>12510.32761409399</v>
+      </c>
+      <c r="I17" s="2" t="n">
+        <v>265.03075</v>
+      </c>
+      <c r="J17" s="3" t="n">
+        <v>46190.88511574074</v>
+      </c>
+      <c r="K17" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
         <v>34.50151836132424</v>
       </c>
-      <c r="B17" s="2" t="n">
+      <c r="B18" s="1" t="n">
         <v>16.28326608417185</v>
       </c>
-      <c r="C17" s="2" t="n">
+      <c r="C18" s="1" t="n">
         <v>47.5049729429652</v>
       </c>
-      <c r="D17" s="2" t="n">
+      <c r="D18" s="1" t="n">
         <v>48.63039547308335</v>
       </c>
-      <c r="E17" s="2" t="n">
+      <c r="E18" s="1" t="n">
         <v>24.91416273803437</v>
       </c>
-      <c r="F17" s="2" t="n">
+      <c r="F18" s="1" t="n">
         <v>42.96185287885277</v>
       </c>
-      <c r="G17" s="2" t="n">
+      <c r="G18" s="1" t="n">
         <v>21.05467413136616</v>
       </c>
-      <c r="H17" s="3" t="n">
+      <c r="H18" s="2" t="n">
         <v>10179.76370213991</v>
       </c>
-      <c r="I17" s="3" t="n">
+      <c r="I18" s="2" t="n">
         <v>385.222</v>
       </c>
-      <c r="J17" s="4" t="n">
+      <c r="J18" s="3" t="n">
         <v>46180.98457175926</v>
       </c>
-      <c r="K17" t="b">
+      <c r="K18" t="b">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K17"/>
+  <autoFilter ref="A1:K18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added explanation for functions, cleaned up code a bit, tried if everything works in new repo (paths, files, packages)
</commit_message>
<xml_diff>
--- a/results_clean.xlsx
+++ b/results_clean.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Results" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results'!$A$1:$K$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results'!$A$1:$K$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -498,34 +498,34 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>16.66845732846889</v>
+        <v>16.44247247215127</v>
       </c>
       <c r="B2" s="1" t="n">
-        <v>14.90057320001673</v>
+        <v>18.088494152856</v>
       </c>
       <c r="C2" s="1" t="n">
-        <v>38.86381047832207</v>
+        <v>36.80253492459242</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>10.03832842036743</v>
+        <v>17.43724048195807</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>28.36416089100964</v>
+        <v>27.02686660047771</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>48.73969842501265</v>
+        <v>49.35198009345779</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>3.060667775754733</v>
+        <v>2.883041734643262</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>13183.1783488889</v>
+        <v>13228.69226245446</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>229.039</v>
+        <v>235.5565</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>46182.78790509259</v>
+        <v>46190.90494212963</v>
       </c>
       <c r="K2" t="b">
         <v>1</v>
@@ -533,34 +533,34 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>13.78471682985224</v>
+        <v>16.66845732846889</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>16.21393024762252</v>
+        <v>14.90057320001673</v>
       </c>
       <c r="C3" s="1" t="n">
-        <v>10.59325996569644</v>
+        <v>38.86381047832207</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>36.06356980491166</v>
+        <v>10.03832842036743</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>36.07082245901849</v>
+        <v>28.36416089100964</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>28.55955393861952</v>
+        <v>48.73969842501265</v>
       </c>
       <c r="G3" s="1" t="n">
-        <v>76.96268176577249</v>
+        <v>3.060667775754733</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>13091.41425410255</v>
+        <v>13183.1783488889</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>234.9595</v>
+        <v>229.039</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>46181.58004629629</v>
+        <v>46182.78790509259</v>
       </c>
       <c r="K3" t="b">
         <v>0</v>
@@ -568,34 +568,34 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>17.79972151146293</v>
+        <v>13.7418009361643</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>17.69341384342146</v>
+        <v>16.52822136788232</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>46.48075530504345</v>
+        <v>35.34117923873767</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>9.328346721716176</v>
+        <v>18.20676275790592</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>32.18668778246325</v>
+        <v>27.8682784770983</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>45.74821535730867</v>
+        <v>49.86328305822444</v>
       </c>
       <c r="G4" s="1" t="n">
-        <v>6.445466519477314</v>
+        <v>1.335201644905327</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>13084.58563732278</v>
+        <v>13178.35622651722</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>234.54925</v>
+        <v>239.3005</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>46182.76752314815</v>
+        <v>46190.89608796296</v>
       </c>
       <c r="K4" t="b">
         <v>0</v>
@@ -603,34 +603,34 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>17.58736126294788</v>
+        <v>13.78471682985224</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>16.45887634010303</v>
+        <v>16.21393024762252</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>47.45352527302221</v>
+        <v>10.59325996569644</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>8.576653324750513</v>
+        <v>36.06356980491166</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>32.82334208094247</v>
+        <v>36.07082245901849</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>46.745392166702</v>
+        <v>28.55955393861952</v>
       </c>
       <c r="G5" s="1" t="n">
-        <v>7.732490961886047</v>
+        <v>76.96268176577249</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>13073.63342736011</v>
+        <v>13091.41425410255</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>230.39875</v>
+        <v>234.9595</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>46182.15122685185</v>
+        <v>46181.58004629629</v>
       </c>
       <c r="K5" t="b">
         <v>0</v>
@@ -638,34 +638,34 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>13.71791013779612</v>
+        <v>17.79972151146293</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>18.10904520314511</v>
+        <v>17.69341384342146</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>10.92071189213304</v>
+        <v>46.48075530504345</v>
       </c>
       <c r="D6" s="1" t="n">
-        <v>36.6622583775164</v>
+        <v>9.328346721716176</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>36.41744258847353</v>
+        <v>32.18668778246325</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>27.51048220857797</v>
+        <v>45.74821535730867</v>
       </c>
       <c r="G6" s="1" t="n">
-        <v>75.74096458387024</v>
+        <v>6.445466519477314</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>13071.57609008536</v>
+        <v>13084.58563732278</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>232.0765</v>
+        <v>234.54925</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>46182.68601851852</v>
+        <v>46182.76752314815</v>
       </c>
       <c r="K6" t="b">
         <v>0</v>
@@ -673,34 +673,34 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>41.8658806151136</v>
+        <v>17.58736126294788</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>15.37870830271605</v>
+        <v>16.45887634010303</v>
       </c>
       <c r="C7" s="1" t="n">
-        <v>23.27808313388434</v>
+        <v>47.45352527302221</v>
       </c>
       <c r="D7" s="1" t="n">
-        <v>17.76876422795642</v>
+        <v>8.576653324750513</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>32.80848986515946</v>
+        <v>32.82334208094247</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>49.56039126315637</v>
+        <v>46.745392166702</v>
       </c>
       <c r="G7" s="1" t="n">
-        <v>4.004847201307703</v>
+        <v>7.732490961886047</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>13041.49585837179</v>
+        <v>13073.63342736011</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>235.48675</v>
+        <v>230.39875</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>46181.61930555556</v>
+        <v>46182.15122685185</v>
       </c>
       <c r="K7" t="b">
         <v>0</v>
@@ -708,34 +708,34 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>15.76699354991495</v>
+        <v>13.71791013779612</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>17.34416185704958</v>
+        <v>18.10904520314511</v>
       </c>
       <c r="C8" s="1" t="n">
-        <v>36.82264430163571</v>
+        <v>10.92071189213304</v>
       </c>
       <c r="D8" s="1" t="n">
-        <v>20.82884517757701</v>
+        <v>36.6622583775164</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>27.54321199229494</v>
+        <v>36.41744258847353</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>43.12916308199385</v>
+        <v>27.51048220857797</v>
       </c>
       <c r="G8" s="1" t="n">
-        <v>4.382860985545683</v>
+        <v>75.74096458387024</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>13039.54099967359</v>
+        <v>13071.57609008536</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>232.88425</v>
+        <v>232.0765</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>46182.61533564814</v>
+        <v>46182.68601851852</v>
       </c>
       <c r="K8" t="b">
         <v>0</v>
@@ -743,34 +743,34 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>12.63807670451446</v>
+        <v>41.8658806151136</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>15.95744954515774</v>
+        <v>15.37870830271605</v>
       </c>
       <c r="C9" s="1" t="n">
-        <v>35.69464860799762</v>
+        <v>23.27808313388434</v>
       </c>
       <c r="D9" s="1" t="n">
-        <v>12.31185540225469</v>
+        <v>17.76876422795642</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>27.67290769582389</v>
+        <v>32.80848986515946</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>39.58733460632672</v>
+        <v>49.56039126315637</v>
       </c>
       <c r="G9" s="1" t="n">
-        <v>15.28166470319942</v>
+        <v>4.004847201307703</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>13030.88753714936</v>
+        <v>13041.49585837179</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>233.16625</v>
+        <v>235.48675</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>46182.59353009259</v>
+        <v>46181.61930555556</v>
       </c>
       <c r="K9" t="b">
         <v>0</v>
@@ -778,34 +778,34 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>16.63370127960484</v>
+        <v>15.76699354991495</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>15.5698375808045</v>
+        <v>17.34416185704958</v>
       </c>
       <c r="C10" s="1" t="n">
-        <v>44.61368353212431</v>
+        <v>36.82264430163571</v>
       </c>
       <c r="D10" s="1" t="n">
-        <v>8.10871062925712</v>
+        <v>20.82884517757701</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>33.48757536800954</v>
+        <v>27.54321199229494</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>47.40549517830886</v>
+        <v>43.12916308199385</v>
       </c>
       <c r="G10" s="1" t="n">
-        <v>6.080468056109986</v>
+        <v>4.382860985545683</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>13024.42830290779</v>
+        <v>13039.54099967359</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>243.60925</v>
+        <v>232.88425</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>46182.57434027778</v>
+        <v>46182.61533564814</v>
       </c>
       <c r="K10" t="b">
         <v>0</v>
@@ -813,34 +813,34 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>17.25260165231997</v>
+        <v>12.63807670451446</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>18.21456551879732</v>
+        <v>15.95744954515774</v>
       </c>
       <c r="C11" s="1" t="n">
-        <v>11.29227638693606</v>
+        <v>35.69464860799762</v>
       </c>
       <c r="D11" s="1" t="n">
-        <v>37.72302288323579</v>
+        <v>12.31185540225469</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>40.53305602737925</v>
+        <v>27.67290769582389</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>30.1222227565979</v>
+        <v>39.58733460632672</v>
       </c>
       <c r="G11" s="1" t="n">
-        <v>73.05607094516266</v>
+        <v>15.28166470319942</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>12999.09867980331</v>
+        <v>13030.88753714936</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>239.53525</v>
+        <v>233.16625</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>46182.60178240741</v>
+        <v>46182.59353009259</v>
       </c>
       <c r="K11" t="b">
         <v>0</v>
@@ -848,34 +848,34 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>43.56368398257163</v>
+        <v>16.63370127960484</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>15.15588461720007</v>
+        <v>15.5698375808045</v>
       </c>
       <c r="C12" s="1" t="n">
-        <v>22.29902711583871</v>
+        <v>44.61368353212431</v>
       </c>
       <c r="D12" s="1" t="n">
-        <v>20.43515019017654</v>
+        <v>8.10871062925712</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>33.88465155652464</v>
+        <v>33.48757536800954</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>48.75409190845778</v>
+        <v>47.40549517830886</v>
       </c>
       <c r="G12" s="1" t="n">
-        <v>3.423824078511241</v>
+        <v>6.080468056109986</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>12985.98554837028</v>
+        <v>13024.42830290779</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>233.1355</v>
+        <v>243.60925</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>46182.52965277778</v>
+        <v>46182.57434027778</v>
       </c>
       <c r="K12" t="b">
         <v>0</v>
@@ -883,34 +883,34 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>17.94757986531874</v>
+        <v>17.25260165231997</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>16.84469598424037</v>
+        <v>18.21456551879732</v>
       </c>
       <c r="C13" s="1" t="n">
-        <v>51.00723850792093</v>
+        <v>11.29227638693606</v>
       </c>
       <c r="D13" s="1" t="n">
-        <v>44.32329678834844</v>
+        <v>37.72302288323579</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>39.51561233856795</v>
+        <v>40.53305602737925</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>34.18006619235404</v>
+        <v>30.1222227565979</v>
       </c>
       <c r="G13" s="1" t="n">
-        <v>49.58832168563249</v>
+        <v>73.05607094516266</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>12926.78503231161</v>
+        <v>12999.09867980331</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>261.9415</v>
+        <v>239.53525</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>46182.52229166667</v>
+        <v>46182.60178240741</v>
       </c>
       <c r="K13" t="b">
         <v>0</v>
@@ -918,34 +918,34 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>11.26262399697765</v>
+        <v>43.56368398257163</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>14.7745708576305</v>
+        <v>15.15588461720007</v>
       </c>
       <c r="C14" s="1" t="n">
-        <v>44.19256877440593</v>
+        <v>22.29902711583871</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>14.75265751951711</v>
+        <v>20.43515019017654</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>31.50532968846312</v>
+        <v>33.88465155652464</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>46.90990440494782</v>
+        <v>48.75409190845778</v>
       </c>
       <c r="G14" s="1" t="n">
-        <v>3.800946599292743</v>
+        <v>3.423824078511241</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>12912.77360106467</v>
+        <v>12985.98554837028</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>234.91</v>
+        <v>233.1355</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>46182.55270833334</v>
+        <v>46182.52965277778</v>
       </c>
       <c r="K14" t="b">
         <v>0</v>
@@ -953,34 +953,34 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>13.33934470733688</v>
+        <v>17.94757986531874</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>16.92409346141374</v>
+        <v>16.84469598424037</v>
       </c>
       <c r="C15" s="1" t="n">
-        <v>36.19215939817842</v>
+        <v>51.00723850792093</v>
       </c>
       <c r="D15" s="1" t="n">
-        <v>14.53122691792867</v>
+        <v>44.32329678834844</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>28.83171218130013</v>
+        <v>39.51561233856795</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>38.49906907960096</v>
+        <v>34.18006619235404</v>
       </c>
       <c r="G15" s="1" t="n">
-        <v>11.29812525550822</v>
+        <v>49.58832168563249</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>12887.47232061737</v>
+        <v>12926.78503231161</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>249.622</v>
+        <v>261.9415</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>46182.563125</v>
+        <v>46182.52229166667</v>
       </c>
       <c r="K15" t="b">
         <v>0</v>
@@ -988,34 +988,34 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>15.626117785012</v>
+        <v>11.26262399697765</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>13.97537155172789</v>
+        <v>14.7745708576305</v>
       </c>
       <c r="C16" s="1" t="n">
-        <v>32.83268303598197</v>
+        <v>44.19256877440593</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>8.326124531530141</v>
+        <v>14.75265751951711</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>34.81057894851994</v>
+        <v>31.50532968846312</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>42.38662545986336</v>
+        <v>46.90990440494782</v>
       </c>
       <c r="G16" s="1" t="n">
-        <v>28.00450830446921</v>
+        <v>3.800946599292743</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>12634.1080121104</v>
+        <v>12912.77360106467</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>267.10675</v>
+        <v>234.91</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>46182.05643518519</v>
+        <v>46182.55270833334</v>
       </c>
       <c r="K16" t="b">
         <v>0</v>
@@ -1023,34 +1023,34 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>15.25529519300532</v>
+        <v>13.33934470733688</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>12.11419195930596</v>
+        <v>16.92409346141374</v>
       </c>
       <c r="C17" s="1" t="n">
-        <v>10.05183024601476</v>
+        <v>36.19215939817842</v>
       </c>
       <c r="D17" s="1" t="n">
-        <v>43.97564648706527</v>
+        <v>14.53122691792867</v>
       </c>
       <c r="E17" s="1" t="n">
-        <v>46.09898454414606</v>
+        <v>28.83171218130013</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>35.73229378624028</v>
+        <v>38.49906907960096</v>
       </c>
       <c r="G17" s="1" t="n">
-        <v>73.32411555469949</v>
+        <v>11.29812525550822</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>12510.32761409399</v>
+        <v>12887.47232061737</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>265.03075</v>
+        <v>249.622</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>46190.88511574074</v>
+        <v>46182.563125</v>
       </c>
       <c r="K17" t="b">
         <v>0</v>
@@ -1058,41 +1058,111 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
+        <v>15.626117785012</v>
+      </c>
+      <c r="B18" s="1" t="n">
+        <v>13.97537155172789</v>
+      </c>
+      <c r="C18" s="1" t="n">
+        <v>32.83268303598197</v>
+      </c>
+      <c r="D18" s="1" t="n">
+        <v>8.326124531530141</v>
+      </c>
+      <c r="E18" s="1" t="n">
+        <v>34.81057894851994</v>
+      </c>
+      <c r="F18" s="1" t="n">
+        <v>42.38662545986336</v>
+      </c>
+      <c r="G18" s="1" t="n">
+        <v>28.00450830446921</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>12634.1080121104</v>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>267.10675</v>
+      </c>
+      <c r="J18" s="3" t="n">
+        <v>46182.05643518519</v>
+      </c>
+      <c r="K18" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n">
+        <v>15.25529519300532</v>
+      </c>
+      <c r="B19" s="1" t="n">
+        <v>12.11419195930596</v>
+      </c>
+      <c r="C19" s="1" t="n">
+        <v>10.05183024601476</v>
+      </c>
+      <c r="D19" s="1" t="n">
+        <v>43.97564648706527</v>
+      </c>
+      <c r="E19" s="1" t="n">
+        <v>46.09898454414606</v>
+      </c>
+      <c r="F19" s="1" t="n">
+        <v>35.73229378624028</v>
+      </c>
+      <c r="G19" s="1" t="n">
+        <v>73.32411555469949</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>12510.32761409399</v>
+      </c>
+      <c r="I19" s="2" t="n">
+        <v>265.03075</v>
+      </c>
+      <c r="J19" s="3" t="n">
+        <v>46190.88511574074</v>
+      </c>
+      <c r="K19" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="n">
         <v>34.50151836132424</v>
       </c>
-      <c r="B18" s="1" t="n">
+      <c r="B20" s="1" t="n">
         <v>16.28326608417185</v>
       </c>
-      <c r="C18" s="1" t="n">
+      <c r="C20" s="1" t="n">
         <v>47.5049729429652</v>
       </c>
-      <c r="D18" s="1" t="n">
+      <c r="D20" s="1" t="n">
         <v>48.63039547308335</v>
       </c>
-      <c r="E18" s="1" t="n">
+      <c r="E20" s="1" t="n">
         <v>24.91416273803437</v>
       </c>
-      <c r="F18" s="1" t="n">
+      <c r="F20" s="1" t="n">
         <v>42.96185287885277</v>
       </c>
-      <c r="G18" s="1" t="n">
+      <c r="G20" s="1" t="n">
         <v>21.05467413136616</v>
       </c>
-      <c r="H18" s="2" t="n">
+      <c r="H20" s="2" t="n">
         <v>10179.76370213991</v>
       </c>
-      <c r="I18" s="2" t="n">
+      <c r="I20" s="2" t="n">
         <v>385.222</v>
       </c>
-      <c r="J18" s="3" t="n">
+      <c r="J20" s="3" t="n">
         <v>46180.98457175926</v>
       </c>
-      <c r="K18" t="b">
+      <c r="K20" t="b">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K18"/>
+  <autoFilter ref="A1:K20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
final runs to show convergence behaviour, plots will be done in excel
</commit_message>
<xml_diff>
--- a/results_clean.xlsx
+++ b/results_clean.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Results" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results'!$A$1:$K$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results'!$A$1:$K$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -533,34 +533,34 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>16.66845732846889</v>
+        <v>13.01443233030595</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>14.90057320001673</v>
+        <v>18.13112408840201</v>
       </c>
       <c r="C3" s="1" t="n">
-        <v>38.86381047832207</v>
+        <v>37.75548919015527</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>10.03832842036743</v>
+        <v>14.27892574916752</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>28.36416089100964</v>
+        <v>26.75657584247617</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>48.73969842501265</v>
+        <v>49.05692901406063</v>
       </c>
       <c r="G3" s="1" t="n">
-        <v>3.060667775754733</v>
+        <v>2.281603344977897</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>13183.1783488889</v>
+        <v>13228.24754910699</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>229.039</v>
+        <v>230.728</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>46182.78790509259</v>
+        <v>46191.56704861111</v>
       </c>
       <c r="K3" t="b">
         <v>0</v>
@@ -568,34 +568,34 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>13.7418009361643</v>
+        <v>17.16371377465441</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>16.52822136788232</v>
+        <v>15.99231491886268</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>35.34117923873767</v>
+        <v>39.23157386520793</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>18.20676275790592</v>
+        <v>13.61961584186429</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>27.8682784770983</v>
+        <v>28.9368777509438</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>49.86328305822444</v>
+        <v>48.54784569666069</v>
       </c>
       <c r="G4" s="1" t="n">
-        <v>1.335201644905327</v>
+        <v>3.910515360055121</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>13178.35622651722</v>
+        <v>13227.84059483939</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>239.3005</v>
+        <v>230.5915</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>46190.89608796296</v>
+        <v>46191.55225694444</v>
       </c>
       <c r="K4" t="b">
         <v>0</v>
@@ -603,34 +603,34 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>13.78471682985224</v>
+        <v>19.26918370175085</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>16.21393024762252</v>
+        <v>18.53959686322831</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>10.59325996569644</v>
+        <v>37.21822333777958</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>36.06356980491166</v>
+        <v>18.52833075714304</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>36.07082245901849</v>
+        <v>29.22384218680862</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>28.55955393861952</v>
+        <v>49.63302089512649</v>
       </c>
       <c r="G5" s="1" t="n">
-        <v>76.96268176577249</v>
+        <v>0.2981457544033443</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>13091.41425410255</v>
+        <v>13225.66443506647</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>234.9595</v>
+        <v>241.96675</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>46181.58004629629</v>
+        <v>46191.52523148148</v>
       </c>
       <c r="K5" t="b">
         <v>0</v>
@@ -638,34 +638,34 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>17.79972151146293</v>
+        <v>43.29101620877238</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>17.69341384342146</v>
+        <v>18.59953952680765</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>46.48075530504345</v>
+        <v>23.15010946523757</v>
       </c>
       <c r="D6" s="1" t="n">
-        <v>9.328346721716176</v>
+        <v>19.22840482381752</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>32.18668778246325</v>
+        <v>32.78021382381935</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>45.74821535730867</v>
+        <v>49.74723688917573</v>
       </c>
       <c r="G6" s="1" t="n">
-        <v>6.445466519477314</v>
+        <v>1.047576765825699</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>13084.58563732278</v>
+        <v>13219.48960370089</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>234.54925</v>
+        <v>234.235</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>46182.76752314815</v>
+        <v>46191.09540509259</v>
       </c>
       <c r="K6" t="b">
         <v>0</v>
@@ -673,34 +673,34 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>17.58736126294788</v>
+        <v>42.37643080134777</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>16.45887634010303</v>
+        <v>18.60747458990511</v>
       </c>
       <c r="C7" s="1" t="n">
-        <v>47.45352527302221</v>
+        <v>22.74876634121728</v>
       </c>
       <c r="D7" s="1" t="n">
-        <v>8.576653324750513</v>
+        <v>19.44701616562086</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>32.82334208094247</v>
+        <v>33.19516442148436</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>46.745392166702</v>
+        <v>50.25994041407482</v>
       </c>
       <c r="G7" s="1" t="n">
-        <v>7.732490961886047</v>
+        <v>0.3907215282105423</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>13073.63342736011</v>
+        <v>13207.45676874419</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>230.39875</v>
+        <v>241.132</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>46182.15122685185</v>
+        <v>46191.11994212963</v>
       </c>
       <c r="K7" t="b">
         <v>0</v>
@@ -708,34 +708,34 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>13.71791013779612</v>
+        <v>15.02360067242675</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>18.10904520314511</v>
+        <v>16.1467157345909</v>
       </c>
       <c r="C8" s="1" t="n">
-        <v>10.92071189213304</v>
+        <v>36.78746845909977</v>
       </c>
       <c r="D8" s="1" t="n">
-        <v>36.6622583775164</v>
+        <v>15.73655408742846</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>36.41744258847353</v>
+        <v>28.86836861186764</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>27.51048220857797</v>
+        <v>48.74357259372626</v>
       </c>
       <c r="G8" s="1" t="n">
-        <v>75.74096458387024</v>
+        <v>1.061718251603305</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>13071.57609008536</v>
+        <v>13206.22443534368</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>232.0765</v>
+        <v>239.017</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>46182.68601851852</v>
+        <v>46191.03938657408</v>
       </c>
       <c r="K8" t="b">
         <v>0</v>
@@ -743,34 +743,34 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>41.8658806151136</v>
+        <v>16.66845732846889</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>15.37870830271605</v>
+        <v>14.90057320001673</v>
       </c>
       <c r="C9" s="1" t="n">
-        <v>23.27808313388434</v>
+        <v>38.86381047832207</v>
       </c>
       <c r="D9" s="1" t="n">
-        <v>17.76876422795642</v>
+        <v>10.03832842036743</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>32.80848986515946</v>
+        <v>28.36416089100964</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>49.56039126315637</v>
+        <v>48.73969842501265</v>
       </c>
       <c r="G9" s="1" t="n">
-        <v>4.004847201307703</v>
+        <v>3.060667775754733</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>13041.49585837179</v>
+        <v>13183.1783488889</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>235.48675</v>
+        <v>229.039</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>46181.61930555556</v>
+        <v>46182.78790509259</v>
       </c>
       <c r="K9" t="b">
         <v>0</v>
@@ -778,34 +778,34 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>15.76699354991495</v>
+        <v>13.7418009361643</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>17.34416185704958</v>
+        <v>16.52822136788232</v>
       </c>
       <c r="C10" s="1" t="n">
-        <v>36.82264430163571</v>
+        <v>35.34117923873767</v>
       </c>
       <c r="D10" s="1" t="n">
-        <v>20.82884517757701</v>
+        <v>18.20676275790592</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>27.54321199229494</v>
+        <v>27.8682784770983</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>43.12916308199385</v>
+        <v>49.86328305822444</v>
       </c>
       <c r="G10" s="1" t="n">
-        <v>4.382860985545683</v>
+        <v>1.335201644905327</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>13039.54099967359</v>
+        <v>13178.35622651722</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>232.88425</v>
+        <v>239.3005</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>46182.61533564814</v>
+        <v>46190.89608796296</v>
       </c>
       <c r="K10" t="b">
         <v>0</v>
@@ -813,34 +813,34 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>12.63807670451446</v>
+        <v>13.78471682985224</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>15.95744954515774</v>
+        <v>16.21393024762252</v>
       </c>
       <c r="C11" s="1" t="n">
-        <v>35.69464860799762</v>
+        <v>10.59325996569644</v>
       </c>
       <c r="D11" s="1" t="n">
-        <v>12.31185540225469</v>
+        <v>36.06356980491166</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>27.67290769582389</v>
+        <v>36.07082245901849</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>39.58733460632672</v>
+        <v>28.55955393861952</v>
       </c>
       <c r="G11" s="1" t="n">
-        <v>15.28166470319942</v>
+        <v>76.96268176577249</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>13030.88753714936</v>
+        <v>13091.41425410255</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>233.16625</v>
+        <v>234.9595</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>46182.59353009259</v>
+        <v>46181.58004629629</v>
       </c>
       <c r="K11" t="b">
         <v>0</v>
@@ -848,34 +848,34 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>16.63370127960484</v>
+        <v>17.79972151146293</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>15.5698375808045</v>
+        <v>17.69341384342146</v>
       </c>
       <c r="C12" s="1" t="n">
-        <v>44.61368353212431</v>
+        <v>46.48075530504345</v>
       </c>
       <c r="D12" s="1" t="n">
-        <v>8.10871062925712</v>
+        <v>9.328346721716176</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>33.48757536800954</v>
+        <v>32.18668778246325</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>47.40549517830886</v>
+        <v>45.74821535730867</v>
       </c>
       <c r="G12" s="1" t="n">
-        <v>6.080468056109986</v>
+        <v>6.445466519477314</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>13024.42830290779</v>
+        <v>13084.58563732278</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>243.60925</v>
+        <v>234.54925</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>46182.57434027778</v>
+        <v>46182.76752314815</v>
       </c>
       <c r="K12" t="b">
         <v>0</v>
@@ -883,34 +883,34 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>17.25260165231997</v>
+        <v>39.3139703377867</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>18.21456551879732</v>
+        <v>17.86931499152951</v>
       </c>
       <c r="C13" s="1" t="n">
-        <v>11.29227638693606</v>
+        <v>43.21703461620231</v>
       </c>
       <c r="D13" s="1" t="n">
-        <v>37.72302288323579</v>
+        <v>45.85382476208808</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>40.53305602737925</v>
+        <v>11.31830513200977</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>30.1222227565979</v>
+        <v>28.1288969572236</v>
       </c>
       <c r="G13" s="1" t="n">
-        <v>73.05607094516266</v>
+        <v>96.36482518351316</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>12999.09867980331</v>
+        <v>13080.22506390762</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>239.53525</v>
+        <v>234.24175</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>46182.60178240741</v>
+        <v>46191.0578587963</v>
       </c>
       <c r="K13" t="b">
         <v>0</v>
@@ -918,34 +918,34 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>43.56368398257163</v>
+        <v>17.58736126294788</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>15.15588461720007</v>
+        <v>16.45887634010303</v>
       </c>
       <c r="C14" s="1" t="n">
-        <v>22.29902711583871</v>
+        <v>47.45352527302221</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>20.43515019017654</v>
+        <v>8.576653324750513</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>33.88465155652464</v>
+        <v>32.82334208094247</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>48.75409190845778</v>
+        <v>46.745392166702</v>
       </c>
       <c r="G14" s="1" t="n">
-        <v>3.423824078511241</v>
+        <v>7.732490961886047</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>12985.98554837028</v>
+        <v>13073.63342736011</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>233.1355</v>
+        <v>230.39875</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>46182.52965277778</v>
+        <v>46182.15122685185</v>
       </c>
       <c r="K14" t="b">
         <v>0</v>
@@ -953,34 +953,34 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>17.94757986531874</v>
+        <v>13.71791013779612</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>16.84469598424037</v>
+        <v>18.10904520314511</v>
       </c>
       <c r="C15" s="1" t="n">
-        <v>51.00723850792093</v>
+        <v>10.92071189213304</v>
       </c>
       <c r="D15" s="1" t="n">
-        <v>44.32329678834844</v>
+        <v>36.6622583775164</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>39.51561233856795</v>
+        <v>36.41744258847353</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>34.18006619235404</v>
+        <v>27.51048220857797</v>
       </c>
       <c r="G15" s="1" t="n">
-        <v>49.58832168563249</v>
+        <v>75.74096458387024</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>12926.78503231161</v>
+        <v>13071.57609008536</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>261.9415</v>
+        <v>232.0765</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>46182.52229166667</v>
+        <v>46182.68601851852</v>
       </c>
       <c r="K15" t="b">
         <v>0</v>
@@ -988,34 +988,34 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>11.26262399697765</v>
+        <v>17.85841600795682</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>14.7745708576305</v>
+        <v>16.5156606710831</v>
       </c>
       <c r="C16" s="1" t="n">
-        <v>44.19256877440593</v>
+        <v>20.15772475639609</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>14.75265751951711</v>
+        <v>40.8248687269072</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>31.50532968846312</v>
+        <v>46.74422061154857</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>46.90990440494782</v>
+        <v>29.81027368968548</v>
       </c>
       <c r="G16" s="1" t="n">
-        <v>3.800946599292743</v>
+        <v>91.11252842958132</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>12912.77360106467</v>
+        <v>13067.12499085083</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>234.91</v>
+        <v>238.96675</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>46182.55270833334</v>
+        <v>46191.07086805555</v>
       </c>
       <c r="K16" t="b">
         <v>0</v>
@@ -1023,34 +1023,34 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>13.33934470733688</v>
+        <v>41.8658806151136</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>16.92409346141374</v>
+        <v>15.37870830271605</v>
       </c>
       <c r="C17" s="1" t="n">
-        <v>36.19215939817842</v>
+        <v>23.27808313388434</v>
       </c>
       <c r="D17" s="1" t="n">
-        <v>14.53122691792867</v>
+        <v>17.76876422795642</v>
       </c>
       <c r="E17" s="1" t="n">
-        <v>28.83171218130013</v>
+        <v>32.80848986515946</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>38.49906907960096</v>
+        <v>49.56039126315637</v>
       </c>
       <c r="G17" s="1" t="n">
-        <v>11.29812525550822</v>
+        <v>4.004847201307703</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>12887.47232061737</v>
+        <v>13041.49585837179</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>249.622</v>
+        <v>235.48675</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>46182.563125</v>
+        <v>46181.61930555556</v>
       </c>
       <c r="K17" t="b">
         <v>0</v>
@@ -1058,34 +1058,34 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>15.626117785012</v>
+        <v>15.76699354991495</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>13.97537155172789</v>
+        <v>17.34416185704958</v>
       </c>
       <c r="C18" s="1" t="n">
-        <v>32.83268303598197</v>
+        <v>36.82264430163571</v>
       </c>
       <c r="D18" s="1" t="n">
-        <v>8.326124531530141</v>
+        <v>20.82884517757701</v>
       </c>
       <c r="E18" s="1" t="n">
-        <v>34.81057894851994</v>
+        <v>27.54321199229494</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>42.38662545986336</v>
+        <v>43.12916308199385</v>
       </c>
       <c r="G18" s="1" t="n">
-        <v>28.00450830446921</v>
+        <v>4.382860985545683</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>12634.1080121104</v>
+        <v>13039.54099967359</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>267.10675</v>
+        <v>232.88425</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>46182.05643518519</v>
+        <v>46182.61533564814</v>
       </c>
       <c r="K18" t="b">
         <v>0</v>
@@ -1093,34 +1093,34 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>15.25529519300532</v>
+        <v>12.63807670451446</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>12.11419195930596</v>
+        <v>15.95744954515774</v>
       </c>
       <c r="C19" s="1" t="n">
-        <v>10.05183024601476</v>
+        <v>35.69464860799762</v>
       </c>
       <c r="D19" s="1" t="n">
-        <v>43.97564648706527</v>
+        <v>12.31185540225469</v>
       </c>
       <c r="E19" s="1" t="n">
-        <v>46.09898454414606</v>
+        <v>27.67290769582389</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>35.73229378624028</v>
+        <v>39.58733460632672</v>
       </c>
       <c r="G19" s="1" t="n">
-        <v>73.32411555469949</v>
+        <v>15.28166470319942</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>12510.32761409399</v>
+        <v>13030.88753714936</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>265.03075</v>
+        <v>233.16625</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>46190.88511574074</v>
+        <v>46182.59353009259</v>
       </c>
       <c r="K19" t="b">
         <v>0</v>
@@ -1128,41 +1128,321 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
+        <v>16.63370127960484</v>
+      </c>
+      <c r="B20" s="1" t="n">
+        <v>15.5698375808045</v>
+      </c>
+      <c r="C20" s="1" t="n">
+        <v>44.61368353212431</v>
+      </c>
+      <c r="D20" s="1" t="n">
+        <v>8.10871062925712</v>
+      </c>
+      <c r="E20" s="1" t="n">
+        <v>33.48757536800954</v>
+      </c>
+      <c r="F20" s="1" t="n">
+        <v>47.40549517830886</v>
+      </c>
+      <c r="G20" s="1" t="n">
+        <v>6.080468056109986</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>13024.42830290779</v>
+      </c>
+      <c r="I20" s="2" t="n">
+        <v>243.60925</v>
+      </c>
+      <c r="J20" s="3" t="n">
+        <v>46182.57434027778</v>
+      </c>
+      <c r="K20" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="n">
+        <v>17.25260165231997</v>
+      </c>
+      <c r="B21" s="1" t="n">
+        <v>18.21456551879732</v>
+      </c>
+      <c r="C21" s="1" t="n">
+        <v>11.29227638693606</v>
+      </c>
+      <c r="D21" s="1" t="n">
+        <v>37.72302288323579</v>
+      </c>
+      <c r="E21" s="1" t="n">
+        <v>40.53305602737925</v>
+      </c>
+      <c r="F21" s="1" t="n">
+        <v>30.1222227565979</v>
+      </c>
+      <c r="G21" s="1" t="n">
+        <v>73.05607094516266</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>12999.09867980331</v>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>239.53525</v>
+      </c>
+      <c r="J21" s="3" t="n">
+        <v>46182.60178240741</v>
+      </c>
+      <c r="K21" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="n">
+        <v>43.56368398257163</v>
+      </c>
+      <c r="B22" s="1" t="n">
+        <v>15.15588461720007</v>
+      </c>
+      <c r="C22" s="1" t="n">
+        <v>22.29902711583871</v>
+      </c>
+      <c r="D22" s="1" t="n">
+        <v>20.43515019017654</v>
+      </c>
+      <c r="E22" s="1" t="n">
+        <v>33.88465155652464</v>
+      </c>
+      <c r="F22" s="1" t="n">
+        <v>48.75409190845778</v>
+      </c>
+      <c r="G22" s="1" t="n">
+        <v>3.423824078511241</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>12985.98554837028</v>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>233.1355</v>
+      </c>
+      <c r="J22" s="3" t="n">
+        <v>46182.52965277778</v>
+      </c>
+      <c r="K22" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n">
+        <v>17.94757986531874</v>
+      </c>
+      <c r="B23" s="1" t="n">
+        <v>16.84469598424037</v>
+      </c>
+      <c r="C23" s="1" t="n">
+        <v>51.00723850792093</v>
+      </c>
+      <c r="D23" s="1" t="n">
+        <v>44.32329678834844</v>
+      </c>
+      <c r="E23" s="1" t="n">
+        <v>39.51561233856795</v>
+      </c>
+      <c r="F23" s="1" t="n">
+        <v>34.18006619235404</v>
+      </c>
+      <c r="G23" s="1" t="n">
+        <v>49.58832168563249</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>12926.78503231161</v>
+      </c>
+      <c r="I23" s="2" t="n">
+        <v>261.9415</v>
+      </c>
+      <c r="J23" s="3" t="n">
+        <v>46182.52229166667</v>
+      </c>
+      <c r="K23" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="n">
+        <v>11.26262399697765</v>
+      </c>
+      <c r="B24" s="1" t="n">
+        <v>14.7745708576305</v>
+      </c>
+      <c r="C24" s="1" t="n">
+        <v>44.19256877440593</v>
+      </c>
+      <c r="D24" s="1" t="n">
+        <v>14.75265751951711</v>
+      </c>
+      <c r="E24" s="1" t="n">
+        <v>31.50532968846312</v>
+      </c>
+      <c r="F24" s="1" t="n">
+        <v>46.90990440494782</v>
+      </c>
+      <c r="G24" s="1" t="n">
+        <v>3.800946599292743</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>12912.77360106467</v>
+      </c>
+      <c r="I24" s="2" t="n">
+        <v>234.91</v>
+      </c>
+      <c r="J24" s="3" t="n">
+        <v>46182.55270833334</v>
+      </c>
+      <c r="K24" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="n">
+        <v>13.33934470733688</v>
+      </c>
+      <c r="B25" s="1" t="n">
+        <v>16.92409346141374</v>
+      </c>
+      <c r="C25" s="1" t="n">
+        <v>36.19215939817842</v>
+      </c>
+      <c r="D25" s="1" t="n">
+        <v>14.53122691792867</v>
+      </c>
+      <c r="E25" s="1" t="n">
+        <v>28.83171218130013</v>
+      </c>
+      <c r="F25" s="1" t="n">
+        <v>38.49906907960096</v>
+      </c>
+      <c r="G25" s="1" t="n">
+        <v>11.29812525550822</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>12887.47232061737</v>
+      </c>
+      <c r="I25" s="2" t="n">
+        <v>249.622</v>
+      </c>
+      <c r="J25" s="3" t="n">
+        <v>46182.563125</v>
+      </c>
+      <c r="K25" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="n">
+        <v>15.626117785012</v>
+      </c>
+      <c r="B26" s="1" t="n">
+        <v>13.97537155172789</v>
+      </c>
+      <c r="C26" s="1" t="n">
+        <v>32.83268303598197</v>
+      </c>
+      <c r="D26" s="1" t="n">
+        <v>8.326124531530141</v>
+      </c>
+      <c r="E26" s="1" t="n">
+        <v>34.81057894851994</v>
+      </c>
+      <c r="F26" s="1" t="n">
+        <v>42.38662545986336</v>
+      </c>
+      <c r="G26" s="1" t="n">
+        <v>28.00450830446921</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>12634.1080121104</v>
+      </c>
+      <c r="I26" s="2" t="n">
+        <v>267.10675</v>
+      </c>
+      <c r="J26" s="3" t="n">
+        <v>46182.05643518519</v>
+      </c>
+      <c r="K26" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n">
+        <v>15.25529519300532</v>
+      </c>
+      <c r="B27" s="1" t="n">
+        <v>12.11419195930596</v>
+      </c>
+      <c r="C27" s="1" t="n">
+        <v>10.05183024601476</v>
+      </c>
+      <c r="D27" s="1" t="n">
+        <v>43.97564648706527</v>
+      </c>
+      <c r="E27" s="1" t="n">
+        <v>46.09898454414606</v>
+      </c>
+      <c r="F27" s="1" t="n">
+        <v>35.73229378624028</v>
+      </c>
+      <c r="G27" s="1" t="n">
+        <v>73.32411555469949</v>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>12510.32761409399</v>
+      </c>
+      <c r="I27" s="2" t="n">
+        <v>265.03075</v>
+      </c>
+      <c r="J27" s="3" t="n">
+        <v>46190.88511574074</v>
+      </c>
+      <c r="K27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="n">
         <v>34.50151836132424</v>
       </c>
-      <c r="B20" s="1" t="n">
+      <c r="B28" s="1" t="n">
         <v>16.28326608417185</v>
       </c>
-      <c r="C20" s="1" t="n">
+      <c r="C28" s="1" t="n">
         <v>47.5049729429652</v>
       </c>
-      <c r="D20" s="1" t="n">
+      <c r="D28" s="1" t="n">
         <v>48.63039547308335</v>
       </c>
-      <c r="E20" s="1" t="n">
+      <c r="E28" s="1" t="n">
         <v>24.91416273803437</v>
       </c>
-      <c r="F20" s="1" t="n">
+      <c r="F28" s="1" t="n">
         <v>42.96185287885277</v>
       </c>
-      <c r="G20" s="1" t="n">
+      <c r="G28" s="1" t="n">
         <v>21.05467413136616</v>
       </c>
-      <c r="H20" s="2" t="n">
+      <c r="H28" s="2" t="n">
         <v>10179.76370213991</v>
       </c>
-      <c r="I20" s="2" t="n">
+      <c r="I28" s="2" t="n">
         <v>385.222</v>
       </c>
-      <c r="J20" s="3" t="n">
+      <c r="J28" s="3" t="n">
         <v>46180.98457175926</v>
       </c>
-      <c r="K20" t="b">
+      <c r="K28" t="b">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K20"/>
+  <autoFilter ref="A1:K28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>